<commit_message>
Commit residual pipeline artifacts from 2026-06-05 run
Recompiled F1 and Golf content data JSONs; updated F1 June 3 PostPlanner
XLSX from format-verification test run.
</commit_message>
<xml_diff>
--- a/F1/postplanner-imports/f1fr-postplanner-2026-06-03.xlsx
+++ b/F1/postplanner-imports/f1fr-postplanner-2026-06-03.xlsx
@@ -478,7 +478,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>06/03/2026  11:57</t>
+          <t>06/03/2026  08:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -495,7 +495,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>06/03/2026  13:27</t>
+          <t>06/03/2026  10:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -511,7 +511,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>06/03/2026  14:57</t>
+          <t>06/03/2026  12:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -528,7 +528,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>06/03/2026  16:27</t>
+          <t>06/03/2026  14:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -547,7 +547,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>06/03/2026  17:57</t>
+          <t>06/03/2026  14:05</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -562,7 +562,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06/03/2026  19:27</t>
+          <t>06/03/2026  17:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">

</xml_diff>